<commit_message>
Add tundish analytics: daily rates, range reports, critical stock, forecast, suggest
- analytics/tundish.py: pure functions for consumption, cover, forecast, requests
- Persian submenu گزارش‌ها / تحلیل تاندیش with date presets and custom range
- PDF sections for the five product goals; CRITICAL_DAYS=3 (configurable)
- Samples aligned so inventory product_name matches material consumption
</commit_message>
<xml_diff>
--- a/samples/01_tank_consumption.xlsx
+++ b/samples/01_tank_consumption.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,25 +526,25 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>T-02</t>
+          <t>T-01</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>سود سوزآور</t>
+          <t>اسید سولفوریک</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>کیلو</t>
+          <t>لیتر</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -552,40 +552,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>خط-B</t>
+          <t>خط-A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>مریم احمدی</t>
+          <t>علی رضایی</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>T-05</t>
+          <t>T-02</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>آب اکسیژنه</t>
+          <t>سود سوزآور</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>لیتر</t>
+          <t>کیلو</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -593,31 +593,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>خط-B</t>
+          <t>خط-A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>حسین کریمی</t>
+          <t>علی رضایی</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>T-06</t>
+          <t>T-02</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>کلر</t>
+          <t>سود سوزآور</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5.5</v>
+        <v>7.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -626,55 +626,260 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>اضطراری</t>
-        </is>
-      </c>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>خط-B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>مریم احمدی</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>T-05</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>آب اکسیژنه</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>لیتر</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>خط-B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>مریم احمدی</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>T-05</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>آب اکسیژنه</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>18</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>لیتر</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>خط-B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>حسین کریمی</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>کلر</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>کیلو</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>اضطراری</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>خط-B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>حسین کریمی</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>کلر</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>کیلو</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>انبار</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>1002</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>مریم احمدی</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>روغن صنعتی</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F10" t="n">
         <v>3</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>انبار</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>مریم احمدی</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>T-10</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>روغن صنعتی</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>لیتر</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add three standard tundish types
</commit_message>
<xml_diff>
--- a/samples/01_tank_consumption.xlsx
+++ b/samples/01_tank_consumption.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,40 +424,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>tundish_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>assignee_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>assignee_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>tundish_id</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>material_name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -471,38 +476,43 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>تاندیش اسلب</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>اسید سولفوریک</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>12.5</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>نوبت صبح</t>
         </is>
@@ -516,38 +526,43 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>تاندیش اسلب</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>اسید سولفوریک</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>11</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -557,38 +572,43 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>تاندیش بلوم</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>سود سوزآور</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>8</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>کیلو</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -598,38 +618,43 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>تاندیش بیلت</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>سود سوزآور</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>7.5</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>کیلو</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -639,38 +664,43 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>تاندیش بلوم</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>1002</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>مریم احمدی</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>آب اکسیژنه</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>20</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -680,38 +710,43 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>تاندیش بیلت</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>1002</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>مریم احمدی</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>آب اکسیژنه</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>18</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -721,38 +756,43 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>تاندیش اسلب</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>1003</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>حسین کریمی</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>کلر</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>5.5</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>کیلو</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>اضطراری</t>
         </is>
@@ -766,38 +806,43 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>تاندیش بلوم</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>1003</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>حسین کریمی</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>کلر</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>6</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>کیلو</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -807,38 +852,43 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>تاندیش بیلت</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>1002</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>مریم احمدی</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>روغن صنعتی</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>3</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -848,38 +898,43 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>تاندیش اسلب</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>1002</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>مریم احمدی</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>روغن صنعتی</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>2.5</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>لیتر</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>